<commit_message>
Resultados de análisis de redes problema6 (1M iteraciones)
</commit_message>
<xml_diff>
--- a/Nuevos DeepWins/Problem6_HierarchicalXOR/Res/Comparativa_10_Neuronas.xlsx
+++ b/Nuevos DeepWins/Problem6_HierarchicalXOR/Res/Comparativa_10_Neuronas.xlsx
@@ -581,42 +581,42 @@
         <v>0.1</v>
       </c>
       <c r="B2" t="n">
-        <v>0.131362</v>
+        <v>0.217309</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>_4_10_1_</t>
+          <t>_4_5_5_1_</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1790733345</v>
+        <v>1790733397</v>
       </c>
       <c r="E2" t="n">
-        <v>52</v>
+        <v>89</v>
       </c>
       <c r="F2" t="n">
         <v>200000</v>
       </c>
       <c r="G2" t="n">
-        <v>0.812958</v>
+        <v>0.686717</v>
       </c>
       <c r="H2" t="n">
-        <v>0.82302</v>
+        <v>0.678218</v>
       </c>
       <c r="I2" t="n">
-        <v>0.817958</v>
+        <v>0.682441</v>
       </c>
       <c r="J2" t="n">
-        <v>0.136797</v>
+        <v>0.225908</v>
       </c>
       <c r="K2" t="n">
-        <v>0.796791</v>
+        <v>0.658768</v>
       </c>
       <c r="L2" t="n">
-        <v>0.768041</v>
+        <v>0.716495</v>
       </c>
       <c r="M2" t="n">
-        <v>0.782152</v>
+        <v>0.68642</v>
       </c>
       <c r="N2" t="n">
         <v>0.2</v>
@@ -652,23 +652,23 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>_4_10_1_1790733345_18.txt</t>
+          <t>_4_5_5_1_1790733397_0.txt</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>[10]</t>
+          <t>[5, 5]</t>
         </is>
       </c>
       <c r="Z2" t="n">
         <v>10</v>
       </c>
       <c r="AA2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
@@ -682,7 +682,7 @@
         <v>0.1</v>
       </c>
       <c r="B3" t="n">
-        <v>0.133193</v>
+        <v>0.125146</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -699,25 +699,25 @@
         <v>200000</v>
       </c>
       <c r="G3" t="n">
-        <v>0.8154979999999999</v>
+        <v>0.821951</v>
       </c>
       <c r="H3" t="n">
-        <v>0.820545</v>
+        <v>0.834158</v>
       </c>
       <c r="I3" t="n">
-        <v>0.818014</v>
+        <v>0.82801</v>
       </c>
       <c r="J3" t="n">
-        <v>0.148404</v>
+        <v>0.136311</v>
       </c>
       <c r="K3" t="n">
-        <v>0.739336</v>
+        <v>0.777251</v>
       </c>
       <c r="L3" t="n">
-        <v>0.8041239999999999</v>
+        <v>0.845361</v>
       </c>
       <c r="M3" t="n">
-        <v>0.77037</v>
+        <v>0.809877</v>
       </c>
       <c r="N3" t="n">
         <v>0.2</v>
@@ -753,7 +753,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>_4_10_1_1790733345_16.txt</t>
+          <t>_4_10_1_1790733345_10.txt</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
@@ -783,7 +783,7 @@
         <v>0.1</v>
       </c>
       <c r="B4" t="n">
-        <v>0.217309</v>
+        <v>0.247666</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -800,25 +800,25 @@
         <v>200000</v>
       </c>
       <c r="G4" t="n">
-        <v>0.686717</v>
+        <v>0.546269</v>
       </c>
       <c r="H4" t="n">
-        <v>0.678218</v>
+        <v>0.679455</v>
       </c>
       <c r="I4" t="n">
-        <v>0.682441</v>
+        <v>0.605626</v>
       </c>
       <c r="J4" t="n">
-        <v>0.225908</v>
+        <v>0.25093</v>
       </c>
       <c r="K4" t="n">
-        <v>0.658768</v>
+        <v>0.5</v>
       </c>
       <c r="L4" t="n">
-        <v>0.716495</v>
+        <v>0.639175</v>
       </c>
       <c r="M4" t="n">
-        <v>0.68642</v>
+        <v>0.561086</v>
       </c>
       <c r="N4" t="n">
         <v>0.2</v>
@@ -854,7 +854,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>_4_5_5_1_1790733397_0.txt</t>
+          <t>_4_5_5_1_1790733397_13.txt</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
@@ -884,42 +884,42 @@
         <v>0.1</v>
       </c>
       <c r="B5" t="n">
-        <v>0.247969</v>
+        <v>0.08407299999999999</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>_4_5_5_1_</t>
+          <t>_4_10_1_</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1790733397</v>
+        <v>1790733345</v>
       </c>
       <c r="E5" t="n">
-        <v>89</v>
+        <v>52</v>
       </c>
       <c r="F5" t="n">
         <v>200000</v>
       </c>
       <c r="G5" t="n">
-        <v>0.526904</v>
+        <v>0.921795</v>
       </c>
       <c r="H5" t="n">
-        <v>0.642327</v>
+        <v>0.889852</v>
       </c>
       <c r="I5" t="n">
-        <v>0.578918</v>
+        <v>0.905542</v>
       </c>
       <c r="J5" t="n">
-        <v>0.250713</v>
+        <v>0.092875</v>
       </c>
       <c r="K5" t="n">
-        <v>0.48583</v>
+        <v>0.895833</v>
       </c>
       <c r="L5" t="n">
-        <v>0.618557</v>
+        <v>0.886598</v>
       </c>
       <c r="M5" t="n">
-        <v>0.544218</v>
+        <v>0.891192</v>
       </c>
       <c r="N5" t="n">
         <v>0.2</v>
@@ -955,28 +955,28 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>_4_5_5_1_1790733397_9.txt</t>
+          <t>_4_10_1_1790733345_2.txt</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>[5, 5]</t>
+          <t>[10]</t>
         </is>
       </c>
       <c r="Z5" t="n">
         <v>10</v>
       </c>
       <c r="AA5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Si</t>
         </is>
       </c>
     </row>
@@ -985,7 +985,7 @@
         <v>0.1</v>
       </c>
       <c r="B6" t="n">
-        <v>0.089249</v>
+        <v>0.126379</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -1002,25 +1002,25 @@
         <v>200000</v>
       </c>
       <c r="G6" t="n">
-        <v>0.903266</v>
+        <v>0.8239610000000001</v>
       </c>
       <c r="H6" t="n">
-        <v>0.889852</v>
+        <v>0.834158</v>
       </c>
       <c r="I6" t="n">
-        <v>0.896509</v>
+        <v>0.829028</v>
       </c>
       <c r="J6" t="n">
-        <v>0.087932</v>
+        <v>0.136189</v>
       </c>
       <c r="K6" t="n">
-        <v>0.927778</v>
+        <v>0.786458</v>
       </c>
       <c r="L6" t="n">
-        <v>0.860825</v>
+        <v>0.778351</v>
       </c>
       <c r="M6" t="n">
-        <v>0.893048</v>
+        <v>0.7823830000000001</v>
       </c>
       <c r="N6" t="n">
         <v>0.2</v>
@@ -1056,7 +1056,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>_4_10_1_1790733345_11.txt</t>
+          <t>_4_10_1_1790733345_12.txt</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
@@ -1077,7 +1077,7 @@
       </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1086,42 +1086,42 @@
         <v>0.1</v>
       </c>
       <c r="B7" t="n">
-        <v>0.23608</v>
+        <v>0.134268</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>_4_5_5_1_</t>
+          <t>_4_10_1_</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1790733397</v>
+        <v>1790733345</v>
       </c>
       <c r="E7" t="n">
-        <v>89</v>
+        <v>52</v>
       </c>
       <c r="F7" t="n">
         <v>200000</v>
       </c>
       <c r="G7" t="n">
-        <v>0.6032110000000001</v>
+        <v>0.800971</v>
       </c>
       <c r="H7" t="n">
-        <v>0.65099</v>
+        <v>0.816832</v>
       </c>
       <c r="I7" t="n">
-        <v>0.62619</v>
+        <v>0.808823</v>
       </c>
       <c r="J7" t="n">
-        <v>0.234687</v>
+        <v>0.141901</v>
       </c>
       <c r="K7" t="n">
-        <v>0.591549</v>
+        <v>0.780749</v>
       </c>
       <c r="L7" t="n">
-        <v>0.649485</v>
+        <v>0.7525770000000001</v>
       </c>
       <c r="M7" t="n">
-        <v>0.619165</v>
+        <v>0.766404</v>
       </c>
       <c r="N7" t="n">
         <v>0.2</v>
@@ -1157,23 +1157,23 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>_4_5_5_1_1790733397_19.txt</t>
+          <t>_4_10_1_1790733345_19.txt</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>[5, 5]</t>
+          <t>[10]</t>
         </is>
       </c>
       <c r="Z7" t="n">
         <v>10</v>
       </c>
       <c r="AA7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB7" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC7" t="inlineStr">
@@ -1187,42 +1187,42 @@
         <v>0.1</v>
       </c>
       <c r="B8" t="n">
-        <v>0.248858</v>
+        <v>0.089249</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>_4_5_5_1_</t>
+          <t>_4_10_1_</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1790733397</v>
+        <v>1790733345</v>
       </c>
       <c r="E8" t="n">
-        <v>89</v>
+        <v>52</v>
       </c>
       <c r="F8" t="n">
         <v>200000</v>
       </c>
       <c r="G8" t="n">
-        <v>0.528133</v>
+        <v>0.903266</v>
       </c>
       <c r="H8" t="n">
-        <v>0.511139</v>
+        <v>0.889852</v>
       </c>
       <c r="I8" t="n">
-        <v>0.519497</v>
+        <v>0.896509</v>
       </c>
       <c r="J8" t="n">
-        <v>0.25115</v>
+        <v>0.087932</v>
       </c>
       <c r="K8" t="n">
-        <v>0.462312</v>
+        <v>0.927778</v>
       </c>
       <c r="L8" t="n">
-        <v>0.474227</v>
+        <v>0.860825</v>
       </c>
       <c r="M8" t="n">
-        <v>0.468193</v>
+        <v>0.893048</v>
       </c>
       <c r="N8" t="n">
         <v>0.2</v>
@@ -1258,28 +1258,28 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>_4_5_5_1_1790733397_6.txt</t>
+          <t>_4_10_1_1790733345_11.txt</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>[5, 5]</t>
+          <t>[10]</t>
         </is>
       </c>
       <c r="Z8" t="n">
         <v>10</v>
       </c>
       <c r="AA8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Si</t>
         </is>
       </c>
     </row>
@@ -1288,42 +1288,42 @@
         <v>0.1</v>
       </c>
       <c r="B9" t="n">
-        <v>0.152629</v>
+        <v>0.23608</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>_4_10_1_</t>
+          <t>_4_5_5_1_</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1790733345</v>
+        <v>1790733397</v>
       </c>
       <c r="E9" t="n">
-        <v>52</v>
+        <v>89</v>
       </c>
       <c r="F9" t="n">
         <v>200000</v>
       </c>
       <c r="G9" t="n">
-        <v>0.780397</v>
+        <v>0.6032110000000001</v>
       </c>
       <c r="H9" t="n">
-        <v>0.778465</v>
+        <v>0.65099</v>
       </c>
       <c r="I9" t="n">
-        <v>0.77943</v>
+        <v>0.62619</v>
       </c>
       <c r="J9" t="n">
-        <v>0.172319</v>
+        <v>0.234687</v>
       </c>
       <c r="K9" t="n">
-        <v>0.748691</v>
+        <v>0.591549</v>
       </c>
       <c r="L9" t="n">
-        <v>0.737113</v>
+        <v>0.649485</v>
       </c>
       <c r="M9" t="n">
-        <v>0.742857</v>
+        <v>0.619165</v>
       </c>
       <c r="N9" t="n">
         <v>0.2</v>
@@ -1359,23 +1359,23 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>_4_10_1_1790733345_6.txt</t>
+          <t>_4_5_5_1_1790733397_19.txt</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>[10]</t>
+          <t>[5, 5]</t>
         </is>
       </c>
       <c r="Z9" t="n">
         <v>10</v>
       </c>
       <c r="AA9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB9" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC9" t="inlineStr">
@@ -1389,7 +1389,7 @@
         <v>0.1</v>
       </c>
       <c r="B10" t="n">
-        <v>0.243926</v>
+        <v>0.17148</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1406,25 +1406,25 @@
         <v>200000</v>
       </c>
       <c r="G10" t="n">
-        <v>0.539033</v>
+        <v>0.727378</v>
       </c>
       <c r="H10" t="n">
-        <v>0.538366</v>
+        <v>0.77599</v>
       </c>
       <c r="I10" t="n">
-        <v>0.5387</v>
+        <v>0.750898</v>
       </c>
       <c r="J10" t="n">
-        <v>0.247216</v>
+        <v>0.187156</v>
       </c>
       <c r="K10" t="n">
-        <v>0.487179</v>
+        <v>0.659292</v>
       </c>
       <c r="L10" t="n">
-        <v>0.489691</v>
+        <v>0.768041</v>
       </c>
       <c r="M10" t="n">
-        <v>0.488432</v>
+        <v>0.709524</v>
       </c>
       <c r="N10" t="n">
         <v>0.2</v>
@@ -1460,7 +1460,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>_4_5_5_1_1790733397_15.txt</t>
+          <t>_4_5_5_1_1790733397_3.txt</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
@@ -1490,7 +1490,7 @@
         <v>0.1</v>
       </c>
       <c r="B11" t="n">
-        <v>0.176646</v>
+        <v>0.249262</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1507,25 +1507,25 @@
         <v>200000</v>
       </c>
       <c r="G11" t="n">
-        <v>0.720253</v>
+        <v>0.52</v>
       </c>
       <c r="H11" t="n">
-        <v>0.7042079999999999</v>
+        <v>0.563119</v>
       </c>
       <c r="I11" t="n">
-        <v>0.71214</v>
+        <v>0.540701</v>
       </c>
       <c r="J11" t="n">
-        <v>0.183729</v>
+        <v>0.251585</v>
       </c>
       <c r="K11" t="n">
-        <v>0.700565</v>
+        <v>0.477876</v>
       </c>
       <c r="L11" t="n">
-        <v>0.639175</v>
+        <v>0.556701</v>
       </c>
       <c r="M11" t="n">
-        <v>0.6684639999999999</v>
+        <v>0.514286</v>
       </c>
       <c r="N11" t="n">
         <v>0.2</v>
@@ -1561,7 +1561,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>_4_5_5_1_1790733397_4.txt</t>
+          <t>_4_5_5_1_1790733397_17.txt</t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
@@ -1591,7 +1591,7 @@
         <v>0.1</v>
       </c>
       <c r="B12" t="n">
-        <v>0.128602</v>
+        <v>0.093891</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1608,25 +1608,25 @@
         <v>200000</v>
       </c>
       <c r="G12" t="n">
-        <v>0.82104</v>
+        <v>0.877928</v>
       </c>
       <c r="H12" t="n">
-        <v>0.840347</v>
+        <v>0.881188</v>
       </c>
       <c r="I12" t="n">
-        <v>0.830581</v>
+        <v>0.879555</v>
       </c>
       <c r="J12" t="n">
-        <v>0.135293</v>
+        <v>0.104515</v>
       </c>
       <c r="K12" t="n">
-        <v>0.804233</v>
+        <v>0.831633</v>
       </c>
       <c r="L12" t="n">
-        <v>0.783505</v>
+        <v>0.840206</v>
       </c>
       <c r="M12" t="n">
-        <v>0.7937340000000001</v>
+        <v>0.835897</v>
       </c>
       <c r="N12" t="n">
         <v>0.2</v>
@@ -1662,7 +1662,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>_4_10_1_1790733345_7.txt</t>
+          <t>_4_10_1_1790733345_9.txt</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="AC12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Si</t>
         </is>
       </c>
     </row>
@@ -1692,42 +1692,42 @@
         <v>0.1</v>
       </c>
       <c r="B13" t="n">
-        <v>0.127037</v>
+        <v>0.249238</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>_4_10_1_</t>
+          <t>_4_5_5_1_</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1790733345</v>
+        <v>1790733397</v>
       </c>
       <c r="E13" t="n">
-        <v>52</v>
+        <v>89</v>
       </c>
       <c r="F13" t="n">
         <v>200000</v>
       </c>
       <c r="G13" t="n">
-        <v>0.822086</v>
+        <v>0.527231</v>
       </c>
       <c r="H13" t="n">
-        <v>0.8292079999999999</v>
+        <v>0.563119</v>
       </c>
       <c r="I13" t="n">
-        <v>0.825632</v>
+        <v>0.544584</v>
       </c>
       <c r="J13" t="n">
-        <v>0.144738</v>
+        <v>0.25162</v>
       </c>
       <c r="K13" t="n">
-        <v>0.773869</v>
+        <v>0.486726</v>
       </c>
       <c r="L13" t="n">
-        <v>0.793814</v>
+        <v>0.56701</v>
       </c>
       <c r="M13" t="n">
-        <v>0.7837150000000001</v>
+        <v>0.523809</v>
       </c>
       <c r="N13" t="n">
         <v>0.2</v>
@@ -1763,23 +1763,23 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>_4_10_1_1790733345_4.txt</t>
+          <t>_4_5_5_1_1790733397_1.txt</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t>[10]</t>
+          <t>[5, 5]</t>
         </is>
       </c>
       <c r="Z13" t="n">
         <v>10</v>
       </c>
       <c r="AA13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC13" t="inlineStr">
@@ -1793,7 +1793,7 @@
         <v>0.1</v>
       </c>
       <c r="B14" t="n">
-        <v>0.210926</v>
+        <v>0.228363</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1810,25 +1810,25 @@
         <v>200000</v>
       </c>
       <c r="G14" t="n">
-        <v>0.660571</v>
+        <v>0.662857</v>
       </c>
       <c r="H14" t="n">
-        <v>0.715347</v>
+        <v>0.574257</v>
       </c>
       <c r="I14" t="n">
-        <v>0.686869</v>
+        <v>0.615385</v>
       </c>
       <c r="J14" t="n">
-        <v>0.20723</v>
+        <v>0.230794</v>
       </c>
       <c r="K14" t="n">
-        <v>0.668203</v>
+        <v>0.630058</v>
       </c>
       <c r="L14" t="n">
-        <v>0.7474229999999999</v>
+        <v>0.561856</v>
       </c>
       <c r="M14" t="n">
-        <v>0.705596</v>
+        <v>0.594005</v>
       </c>
       <c r="N14" t="n">
         <v>0.2</v>
@@ -1864,7 +1864,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>_4_5_5_1_1790733397_7.txt</t>
+          <t>_4_5_5_1_1790733397_10.txt</t>
         </is>
       </c>
       <c r="Y14" t="inlineStr">
@@ -1894,7 +1894,7 @@
         <v>0.1</v>
       </c>
       <c r="B15" t="n">
-        <v>0.081584</v>
+        <v>0.119723</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1911,25 +1911,25 @@
         <v>200000</v>
       </c>
       <c r="G15" t="n">
-        <v>0.91067</v>
+        <v>0.819512</v>
       </c>
       <c r="H15" t="n">
-        <v>0.908416</v>
+        <v>0.831683</v>
       </c>
       <c r="I15" t="n">
-        <v>0.909542</v>
+        <v>0.825553</v>
       </c>
       <c r="J15" t="n">
-        <v>0.082622</v>
+        <v>0.126751</v>
       </c>
       <c r="K15" t="n">
-        <v>0.939891</v>
+        <v>0.820106</v>
       </c>
       <c r="L15" t="n">
-        <v>0.886598</v>
+        <v>0.798969</v>
       </c>
       <c r="M15" t="n">
-        <v>0.912467</v>
+        <v>0.809399</v>
       </c>
       <c r="N15" t="n">
         <v>0.2</v>
@@ -1965,7 +1965,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>_4_10_1_1790733345_8.txt</t>
+          <t>_4_10_1_1790733345_3.txt</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="AC15" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1995,7 +1995,7 @@
         <v>0.1</v>
       </c>
       <c r="B16" t="n">
-        <v>0.249238</v>
+        <v>0.243926</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -2012,25 +2012,25 @@
         <v>200000</v>
       </c>
       <c r="G16" t="n">
-        <v>0.527231</v>
+        <v>0.539033</v>
       </c>
       <c r="H16" t="n">
-        <v>0.563119</v>
+        <v>0.538366</v>
       </c>
       <c r="I16" t="n">
-        <v>0.544584</v>
+        <v>0.5387</v>
       </c>
       <c r="J16" t="n">
-        <v>0.25162</v>
+        <v>0.247216</v>
       </c>
       <c r="K16" t="n">
-        <v>0.486726</v>
+        <v>0.487179</v>
       </c>
       <c r="L16" t="n">
-        <v>0.56701</v>
+        <v>0.489691</v>
       </c>
       <c r="M16" t="n">
-        <v>0.523809</v>
+        <v>0.488432</v>
       </c>
       <c r="N16" t="n">
         <v>0.2</v>
@@ -2066,7 +2066,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>_4_5_5_1_1790733397_1.txt</t>
+          <t>_4_5_5_1_1790733397_15.txt</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
@@ -2096,42 +2096,42 @@
         <v>0.1</v>
       </c>
       <c r="B17" t="n">
-        <v>0.13385</v>
+        <v>0.210926</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>_4_10_1_</t>
+          <t>_4_5_5_1_</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>1790733345</v>
+        <v>1790733397</v>
       </c>
       <c r="E17" t="n">
-        <v>52</v>
+        <v>89</v>
       </c>
       <c r="F17" t="n">
         <v>200000</v>
       </c>
       <c r="G17" t="n">
-        <v>0.81715</v>
+        <v>0.660571</v>
       </c>
       <c r="H17" t="n">
-        <v>0.80198</v>
+        <v>0.715347</v>
       </c>
       <c r="I17" t="n">
-        <v>0.809494</v>
+        <v>0.686869</v>
       </c>
       <c r="J17" t="n">
-        <v>0.134381</v>
+        <v>0.20723</v>
       </c>
       <c r="K17" t="n">
-        <v>0.801047</v>
+        <v>0.668203</v>
       </c>
       <c r="L17" t="n">
-        <v>0.78866</v>
+        <v>0.7474229999999999</v>
       </c>
       <c r="M17" t="n">
-        <v>0.794805</v>
+        <v>0.705596</v>
       </c>
       <c r="N17" t="n">
         <v>0.2</v>
@@ -2167,23 +2167,23 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>_4_10_1_1790733345_14.txt</t>
+          <t>_4_5_5_1_1790733397_7.txt</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>[10]</t>
+          <t>[5, 5]</t>
         </is>
       </c>
       <c r="Z17" t="n">
         <v>10</v>
       </c>
       <c r="AA17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB17" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC17" t="inlineStr">
@@ -2197,42 +2197,42 @@
         <v>0.1</v>
       </c>
       <c r="B18" t="n">
-        <v>0.247666</v>
+        <v>0.128602</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>_4_5_5_1_</t>
+          <t>_4_10_1_</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>1790733397</v>
+        <v>1790733345</v>
       </c>
       <c r="E18" t="n">
-        <v>89</v>
+        <v>52</v>
       </c>
       <c r="F18" t="n">
         <v>200000</v>
       </c>
       <c r="G18" t="n">
-        <v>0.546269</v>
+        <v>0.82104</v>
       </c>
       <c r="H18" t="n">
-        <v>0.679455</v>
+        <v>0.840347</v>
       </c>
       <c r="I18" t="n">
-        <v>0.605626</v>
+        <v>0.830581</v>
       </c>
       <c r="J18" t="n">
-        <v>0.25093</v>
+        <v>0.135293</v>
       </c>
       <c r="K18" t="n">
-        <v>0.5</v>
+        <v>0.804233</v>
       </c>
       <c r="L18" t="n">
-        <v>0.639175</v>
+        <v>0.783505</v>
       </c>
       <c r="M18" t="n">
-        <v>0.561086</v>
+        <v>0.7937340000000001</v>
       </c>
       <c r="N18" t="n">
         <v>0.2</v>
@@ -2268,23 +2268,23 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>_4_5_5_1_1790733397_13.txt</t>
+          <t>_4_10_1_1790733345_7.txt</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>[5, 5]</t>
+          <t>[10]</t>
         </is>
       </c>
       <c r="Z18" t="n">
         <v>10</v>
       </c>
       <c r="AA18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB18" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC18" t="inlineStr">
@@ -2298,7 +2298,7 @@
         <v>0.1</v>
       </c>
       <c r="B19" t="n">
-        <v>0.249019</v>
+        <v>0.249287</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2315,25 +2315,25 @@
         <v>200000</v>
       </c>
       <c r="G19" t="n">
-        <v>0.524076</v>
+        <v>0.522753</v>
       </c>
       <c r="H19" t="n">
-        <v>0.5792079999999999</v>
+        <v>0.582921</v>
       </c>
       <c r="I19" t="n">
-        <v>0.550265</v>
+        <v>0.5512</v>
       </c>
       <c r="J19" t="n">
-        <v>0.251018</v>
+        <v>0.251687</v>
       </c>
       <c r="K19" t="n">
-        <v>0.491071</v>
+        <v>0.487069</v>
       </c>
       <c r="L19" t="n">
-        <v>0.56701</v>
+        <v>0.582474</v>
       </c>
       <c r="M19" t="n">
-        <v>0.526316</v>
+        <v>0.530516</v>
       </c>
       <c r="N19" t="n">
         <v>0.2</v>
@@ -2369,7 +2369,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>_4_5_5_1_1790733397_16.txt</t>
+          <t>_4_5_5_1_1790733397_14.txt</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
@@ -2399,7 +2399,7 @@
         <v>0.1</v>
       </c>
       <c r="B20" t="n">
-        <v>0.134958</v>
+        <v>0.081584</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2416,25 +2416,25 @@
         <v>200000</v>
       </c>
       <c r="G20" t="n">
-        <v>0.812422</v>
+        <v>0.91067</v>
       </c>
       <c r="H20" t="n">
-        <v>0.809406</v>
+        <v>0.908416</v>
       </c>
       <c r="I20" t="n">
-        <v>0.810911</v>
+        <v>0.909542</v>
       </c>
       <c r="J20" t="n">
-        <v>0.137102</v>
+        <v>0.082622</v>
       </c>
       <c r="K20" t="n">
-        <v>0.77</v>
+        <v>0.939891</v>
       </c>
       <c r="L20" t="n">
-        <v>0.793814</v>
+        <v>0.886598</v>
       </c>
       <c r="M20" t="n">
-        <v>0.781726</v>
+        <v>0.912467</v>
       </c>
       <c r="N20" t="n">
         <v>0.2</v>
@@ -2470,7 +2470,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>_4_10_1_1790733345_13.txt</t>
+          <t>_4_10_1_1790733345_8.txt</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
@@ -2491,7 +2491,7 @@
       </c>
       <c r="AC20" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Si</t>
         </is>
       </c>
     </row>
@@ -2500,7 +2500,7 @@
         <v>0.1</v>
       </c>
       <c r="B21" t="n">
-        <v>0.17148</v>
+        <v>0.248858</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2517,25 +2517,25 @@
         <v>200000</v>
       </c>
       <c r="G21" t="n">
-        <v>0.727378</v>
+        <v>0.528133</v>
       </c>
       <c r="H21" t="n">
-        <v>0.77599</v>
+        <v>0.511139</v>
       </c>
       <c r="I21" t="n">
-        <v>0.750898</v>
+        <v>0.519497</v>
       </c>
       <c r="J21" t="n">
-        <v>0.187156</v>
+        <v>0.25115</v>
       </c>
       <c r="K21" t="n">
-        <v>0.659292</v>
+        <v>0.462312</v>
       </c>
       <c r="L21" t="n">
-        <v>0.768041</v>
+        <v>0.474227</v>
       </c>
       <c r="M21" t="n">
-        <v>0.709524</v>
+        <v>0.468193</v>
       </c>
       <c r="N21" t="n">
         <v>0.2</v>
@@ -2571,7 +2571,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>_4_5_5_1_1790733397_3.txt</t>
+          <t>_4_5_5_1_1790733397_6.txt</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
@@ -2601,42 +2601,42 @@
         <v>0.1</v>
       </c>
       <c r="B22" t="n">
-        <v>0.222716</v>
+        <v>0.13385</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>_4_5_5_1_</t>
+          <t>_4_10_1_</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>1790733397</v>
+        <v>1790733345</v>
       </c>
       <c r="E22" t="n">
-        <v>89</v>
+        <v>52</v>
       </c>
       <c r="F22" t="n">
         <v>200000</v>
       </c>
       <c r="G22" t="n">
-        <v>0.658838</v>
+        <v>0.81715</v>
       </c>
       <c r="H22" t="n">
-        <v>0.659653</v>
+        <v>0.80198</v>
       </c>
       <c r="I22" t="n">
-        <v>0.659246</v>
+        <v>0.809494</v>
       </c>
       <c r="J22" t="n">
-        <v>0.232232</v>
+        <v>0.134381</v>
       </c>
       <c r="K22" t="n">
-        <v>0.63587</v>
+        <v>0.801047</v>
       </c>
       <c r="L22" t="n">
-        <v>0.603093</v>
+        <v>0.78866</v>
       </c>
       <c r="M22" t="n">
-        <v>0.619048</v>
+        <v>0.794805</v>
       </c>
       <c r="N22" t="n">
         <v>0.2</v>
@@ -2672,23 +2672,23 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>_4_5_5_1_1790733397_8.txt</t>
+          <t>_4_10_1_1790733345_14.txt</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>[5, 5]</t>
+          <t>[10]</t>
         </is>
       </c>
       <c r="Z22" t="n">
         <v>10</v>
       </c>
       <c r="AA22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB22" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC22" t="inlineStr">
@@ -2702,7 +2702,7 @@
         <v>0.1</v>
       </c>
       <c r="B23" t="n">
-        <v>0.129223</v>
+        <v>0.135044</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -2719,25 +2719,25 @@
         <v>200000</v>
       </c>
       <c r="G23" t="n">
-        <v>0.805861</v>
+        <v>0.805</v>
       </c>
       <c r="H23" t="n">
-        <v>0.816832</v>
+        <v>0.79703</v>
       </c>
       <c r="I23" t="n">
-        <v>0.8113089999999999</v>
+        <v>0.800995</v>
       </c>
       <c r="J23" t="n">
-        <v>0.141638</v>
+        <v>0.147561</v>
       </c>
       <c r="K23" t="n">
-        <v>0.765854</v>
+        <v>0.787879</v>
       </c>
       <c r="L23" t="n">
-        <v>0.8092780000000001</v>
+        <v>0.8041239999999999</v>
       </c>
       <c r="M23" t="n">
-        <v>0.786967</v>
+        <v>0.795918</v>
       </c>
       <c r="N23" t="n">
         <v>0.2</v>
@@ -2773,7 +2773,7 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>_4_10_1_1790733345_0.txt</t>
+          <t>_4_10_1_1790733345_1.txt</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
@@ -2803,42 +2803,42 @@
         <v>0.1</v>
       </c>
       <c r="B24" t="n">
-        <v>0.249262</v>
+        <v>0.133193</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>_4_5_5_1_</t>
+          <t>_4_10_1_</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>1790733397</v>
+        <v>1790733345</v>
       </c>
       <c r="E24" t="n">
-        <v>89</v>
+        <v>52</v>
       </c>
       <c r="F24" t="n">
         <v>200000</v>
       </c>
       <c r="G24" t="n">
-        <v>0.52</v>
+        <v>0.8154979999999999</v>
       </c>
       <c r="H24" t="n">
-        <v>0.563119</v>
+        <v>0.820545</v>
       </c>
       <c r="I24" t="n">
-        <v>0.540701</v>
+        <v>0.818014</v>
       </c>
       <c r="J24" t="n">
-        <v>0.251585</v>
+        <v>0.148404</v>
       </c>
       <c r="K24" t="n">
-        <v>0.477876</v>
+        <v>0.739336</v>
       </c>
       <c r="L24" t="n">
-        <v>0.556701</v>
+        <v>0.8041239999999999</v>
       </c>
       <c r="M24" t="n">
-        <v>0.514286</v>
+        <v>0.77037</v>
       </c>
       <c r="N24" t="n">
         <v>0.2</v>
@@ -2874,23 +2874,23 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>_4_5_5_1_1790733397_17.txt</t>
+          <t>_4_10_1_1790733345_16.txt</t>
         </is>
       </c>
       <c r="Y24" t="inlineStr">
         <is>
-          <t>[5, 5]</t>
+          <t>[10]</t>
         </is>
       </c>
       <c r="Z24" t="n">
         <v>10</v>
       </c>
       <c r="AA24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB24" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC24" t="inlineStr">
@@ -2904,42 +2904,42 @@
         <v>0.1</v>
       </c>
       <c r="B25" t="n">
-        <v>0.126379</v>
+        <v>0.244959</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>_4_10_1_</t>
+          <t>_4_5_5_1_</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>1790733345</v>
+        <v>1790733397</v>
       </c>
       <c r="E25" t="n">
-        <v>52</v>
+        <v>89</v>
       </c>
       <c r="F25" t="n">
         <v>200000</v>
       </c>
       <c r="G25" t="n">
-        <v>0.8239610000000001</v>
+        <v>0.590835</v>
       </c>
       <c r="H25" t="n">
-        <v>0.834158</v>
+        <v>0.446782</v>
       </c>
       <c r="I25" t="n">
-        <v>0.829028</v>
+        <v>0.508809</v>
       </c>
       <c r="J25" t="n">
-        <v>0.136189</v>
+        <v>0.247204</v>
       </c>
       <c r="K25" t="n">
-        <v>0.786458</v>
+        <v>0.550336</v>
       </c>
       <c r="L25" t="n">
-        <v>0.778351</v>
+        <v>0.42268</v>
       </c>
       <c r="M25" t="n">
-        <v>0.7823830000000001</v>
+        <v>0.478134</v>
       </c>
       <c r="N25" t="n">
         <v>0.2</v>
@@ -2975,23 +2975,23 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>_4_10_1_1790733345_12.txt</t>
+          <t>_4_5_5_1_1790733397_5.txt</t>
         </is>
       </c>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>[10]</t>
+          <t>[5, 5]</t>
         </is>
       </c>
       <c r="Z25" t="n">
         <v>10</v>
       </c>
       <c r="AA25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB25" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC25" t="inlineStr">
@@ -3005,42 +3005,42 @@
         <v>0.1</v>
       </c>
       <c r="B26" t="n">
-        <v>0.119723</v>
+        <v>0.222716</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>_4_10_1_</t>
+          <t>_4_5_5_1_</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>1790733345</v>
+        <v>1790733397</v>
       </c>
       <c r="E26" t="n">
-        <v>52</v>
+        <v>89</v>
       </c>
       <c r="F26" t="n">
         <v>200000</v>
       </c>
       <c r="G26" t="n">
-        <v>0.819512</v>
+        <v>0.658838</v>
       </c>
       <c r="H26" t="n">
-        <v>0.831683</v>
+        <v>0.659653</v>
       </c>
       <c r="I26" t="n">
-        <v>0.825553</v>
+        <v>0.659246</v>
       </c>
       <c r="J26" t="n">
-        <v>0.126751</v>
+        <v>0.232232</v>
       </c>
       <c r="K26" t="n">
-        <v>0.820106</v>
+        <v>0.63587</v>
       </c>
       <c r="L26" t="n">
-        <v>0.798969</v>
+        <v>0.603093</v>
       </c>
       <c r="M26" t="n">
-        <v>0.809399</v>
+        <v>0.619048</v>
       </c>
       <c r="N26" t="n">
         <v>0.2</v>
@@ -3076,23 +3076,23 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>_4_10_1_1790733345_3.txt</t>
+          <t>_4_5_5_1_1790733397_8.txt</t>
         </is>
       </c>
       <c r="Y26" t="inlineStr">
         <is>
-          <t>[10]</t>
+          <t>[5, 5]</t>
         </is>
       </c>
       <c r="Z26" t="n">
         <v>10</v>
       </c>
       <c r="AA26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB26" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC26" t="inlineStr">
@@ -3207,42 +3207,42 @@
         <v>0.1</v>
       </c>
       <c r="B28" t="n">
-        <v>0.249287</v>
+        <v>0.127037</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>_4_5_5_1_</t>
+          <t>_4_10_1_</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>1790733397</v>
+        <v>1790733345</v>
       </c>
       <c r="E28" t="n">
-        <v>89</v>
+        <v>52</v>
       </c>
       <c r="F28" t="n">
         <v>200000</v>
       </c>
       <c r="G28" t="n">
-        <v>0.522753</v>
+        <v>0.822086</v>
       </c>
       <c r="H28" t="n">
-        <v>0.582921</v>
+        <v>0.8292079999999999</v>
       </c>
       <c r="I28" t="n">
-        <v>0.5512</v>
+        <v>0.825632</v>
       </c>
       <c r="J28" t="n">
-        <v>0.251687</v>
+        <v>0.144738</v>
       </c>
       <c r="K28" t="n">
-        <v>0.487069</v>
+        <v>0.773869</v>
       </c>
       <c r="L28" t="n">
-        <v>0.582474</v>
+        <v>0.793814</v>
       </c>
       <c r="M28" t="n">
-        <v>0.530516</v>
+        <v>0.7837150000000001</v>
       </c>
       <c r="N28" t="n">
         <v>0.2</v>
@@ -3278,23 +3278,23 @@
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>_4_5_5_1_1790733397_14.txt</t>
+          <t>_4_10_1_1790733345_4.txt</t>
         </is>
       </c>
       <c r="Y28" t="inlineStr">
         <is>
-          <t>[5, 5]</t>
+          <t>[10]</t>
         </is>
       </c>
       <c r="Z28" t="n">
         <v>10</v>
       </c>
       <c r="AA28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB28" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC28" t="inlineStr">
@@ -3308,42 +3308,42 @@
         <v>0.1</v>
       </c>
       <c r="B29" t="n">
-        <v>0.121098</v>
+        <v>0.249019</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>_4_10_1_</t>
+          <t>_4_5_5_1_</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>1790733345</v>
+        <v>1790733397</v>
       </c>
       <c r="E29" t="n">
-        <v>52</v>
+        <v>89</v>
       </c>
       <c r="F29" t="n">
         <v>200000</v>
       </c>
       <c r="G29" t="n">
-        <v>0.826406</v>
+        <v>0.524076</v>
       </c>
       <c r="H29" t="n">
-        <v>0.836634</v>
+        <v>0.5792079999999999</v>
       </c>
       <c r="I29" t="n">
-        <v>0.831488</v>
+        <v>0.550265</v>
       </c>
       <c r="J29" t="n">
-        <v>0.131535</v>
+        <v>0.251018</v>
       </c>
       <c r="K29" t="n">
-        <v>0.808511</v>
+        <v>0.491071</v>
       </c>
       <c r="L29" t="n">
-        <v>0.783505</v>
+        <v>0.56701</v>
       </c>
       <c r="M29" t="n">
-        <v>0.795812</v>
+        <v>0.526316</v>
       </c>
       <c r="N29" t="n">
         <v>0.2</v>
@@ -3379,23 +3379,23 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>_4_10_1_1790733345_15.txt</t>
+          <t>_4_5_5_1_1790733397_16.txt</t>
         </is>
       </c>
       <c r="Y29" t="inlineStr">
         <is>
-          <t>[10]</t>
+          <t>[5, 5]</t>
         </is>
       </c>
       <c r="Z29" t="n">
         <v>10</v>
       </c>
       <c r="AA29" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB29" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC29" t="inlineStr">
@@ -3409,7 +3409,7 @@
         <v>0.1</v>
       </c>
       <c r="B30" t="n">
-        <v>0.228363</v>
+        <v>0.24342</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -3426,25 +3426,25 @@
         <v>200000</v>
       </c>
       <c r="G30" t="n">
-        <v>0.662857</v>
+        <v>0.550864</v>
       </c>
       <c r="H30" t="n">
-        <v>0.574257</v>
+        <v>0.710396</v>
       </c>
       <c r="I30" t="n">
-        <v>0.615385</v>
+        <v>0.620541</v>
       </c>
       <c r="J30" t="n">
-        <v>0.230794</v>
+        <v>0.245001</v>
       </c>
       <c r="K30" t="n">
-        <v>0.630058</v>
+        <v>0.523077</v>
       </c>
       <c r="L30" t="n">
-        <v>0.561856</v>
+        <v>0.701031</v>
       </c>
       <c r="M30" t="n">
-        <v>0.594005</v>
+        <v>0.599119</v>
       </c>
       <c r="N30" t="n">
         <v>0.2</v>
@@ -3480,7 +3480,7 @@
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>_4_5_5_1_1790733397_10.txt</t>
+          <t>_4_5_5_1_1790733397_12.txt</t>
         </is>
       </c>
       <c r="Y30" t="inlineStr">
@@ -3510,7 +3510,7 @@
         <v>0.1</v>
       </c>
       <c r="B31" t="n">
-        <v>0.135044</v>
+        <v>0.152629</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -3527,25 +3527,25 @@
         <v>200000</v>
       </c>
       <c r="G31" t="n">
-        <v>0.805</v>
+        <v>0.780397</v>
       </c>
       <c r="H31" t="n">
-        <v>0.79703</v>
+        <v>0.778465</v>
       </c>
       <c r="I31" t="n">
-        <v>0.800995</v>
+        <v>0.77943</v>
       </c>
       <c r="J31" t="n">
-        <v>0.147561</v>
+        <v>0.172319</v>
       </c>
       <c r="K31" t="n">
-        <v>0.787879</v>
+        <v>0.748691</v>
       </c>
       <c r="L31" t="n">
-        <v>0.8041239999999999</v>
+        <v>0.737113</v>
       </c>
       <c r="M31" t="n">
-        <v>0.795918</v>
+        <v>0.742857</v>
       </c>
       <c r="N31" t="n">
         <v>0.2</v>
@@ -3581,7 +3581,7 @@
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>_4_10_1_1790733345_1.txt</t>
+          <t>_4_10_1_1790733345_6.txt</t>
         </is>
       </c>
       <c r="Y31" t="inlineStr">
@@ -3611,42 +3611,42 @@
         <v>0.1</v>
       </c>
       <c r="B32" t="n">
-        <v>0.125146</v>
+        <v>0.247969</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>_4_10_1_</t>
+          <t>_4_5_5_1_</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>1790733345</v>
+        <v>1790733397</v>
       </c>
       <c r="E32" t="n">
-        <v>52</v>
+        <v>89</v>
       </c>
       <c r="F32" t="n">
         <v>200000</v>
       </c>
       <c r="G32" t="n">
-        <v>0.821951</v>
+        <v>0.526904</v>
       </c>
       <c r="H32" t="n">
-        <v>0.834158</v>
+        <v>0.642327</v>
       </c>
       <c r="I32" t="n">
-        <v>0.82801</v>
+        <v>0.578918</v>
       </c>
       <c r="J32" t="n">
-        <v>0.136311</v>
+        <v>0.250713</v>
       </c>
       <c r="K32" t="n">
-        <v>0.777251</v>
+        <v>0.48583</v>
       </c>
       <c r="L32" t="n">
-        <v>0.845361</v>
+        <v>0.618557</v>
       </c>
       <c r="M32" t="n">
-        <v>0.809877</v>
+        <v>0.544218</v>
       </c>
       <c r="N32" t="n">
         <v>0.2</v>
@@ -3682,23 +3682,23 @@
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>_4_10_1_1790733345_10.txt</t>
+          <t>_4_5_5_1_1790733397_9.txt</t>
         </is>
       </c>
       <c r="Y32" t="inlineStr">
         <is>
-          <t>[10]</t>
+          <t>[5, 5]</t>
         </is>
       </c>
       <c r="Z32" t="n">
         <v>10</v>
       </c>
       <c r="AA32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB32" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC32" t="inlineStr">
@@ -3712,7 +3712,7 @@
         <v>0.1</v>
       </c>
       <c r="B33" t="n">
-        <v>0.244959</v>
+        <v>0.22867</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -3729,25 +3729,25 @@
         <v>200000</v>
       </c>
       <c r="G33" t="n">
-        <v>0.590835</v>
+        <v>0.655797</v>
       </c>
       <c r="H33" t="n">
-        <v>0.446782</v>
+        <v>0.67203</v>
       </c>
       <c r="I33" t="n">
-        <v>0.508809</v>
+        <v>0.663814</v>
       </c>
       <c r="J33" t="n">
-        <v>0.247204</v>
+        <v>0.229602</v>
       </c>
       <c r="K33" t="n">
-        <v>0.550336</v>
+        <v>0.625592</v>
       </c>
       <c r="L33" t="n">
-        <v>0.42268</v>
+        <v>0.680412</v>
       </c>
       <c r="M33" t="n">
-        <v>0.478134</v>
+        <v>0.651852</v>
       </c>
       <c r="N33" t="n">
         <v>0.2</v>
@@ -3783,7 +3783,7 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>_4_5_5_1_1790733397_5.txt</t>
+          <t>_4_5_5_1_1790733397_11.txt</t>
         </is>
       </c>
       <c r="Y33" t="inlineStr">
@@ -3813,7 +3813,7 @@
         <v>0.1</v>
       </c>
       <c r="B34" t="n">
-        <v>0.24342</v>
+        <v>0.210196</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -3830,25 +3830,25 @@
         <v>200000</v>
       </c>
       <c r="G34" t="n">
-        <v>0.550864</v>
+        <v>0.666253</v>
       </c>
       <c r="H34" t="n">
-        <v>0.710396</v>
+        <v>0.664604</v>
       </c>
       <c r="I34" t="n">
-        <v>0.620541</v>
+        <v>0.665428</v>
       </c>
       <c r="J34" t="n">
-        <v>0.245001</v>
+        <v>0.205773</v>
       </c>
       <c r="K34" t="n">
-        <v>0.523077</v>
+        <v>0.6769230000000001</v>
       </c>
       <c r="L34" t="n">
-        <v>0.701031</v>
+        <v>0.680412</v>
       </c>
       <c r="M34" t="n">
-        <v>0.599119</v>
+        <v>0.678663</v>
       </c>
       <c r="N34" t="n">
         <v>0.2</v>
@@ -3884,7 +3884,7 @@
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>_4_5_5_1_1790733397_12.txt</t>
+          <t>_4_5_5_1_1790733397_2.txt</t>
         </is>
       </c>
       <c r="Y34" t="inlineStr">
@@ -3914,7 +3914,7 @@
         <v>0.1</v>
       </c>
       <c r="B35" t="n">
-        <v>0.08407299999999999</v>
+        <v>0.134958</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -3931,25 +3931,25 @@
         <v>200000</v>
       </c>
       <c r="G35" t="n">
-        <v>0.921795</v>
+        <v>0.812422</v>
       </c>
       <c r="H35" t="n">
-        <v>0.889852</v>
+        <v>0.809406</v>
       </c>
       <c r="I35" t="n">
-        <v>0.905542</v>
+        <v>0.810911</v>
       </c>
       <c r="J35" t="n">
-        <v>0.092875</v>
+        <v>0.137102</v>
       </c>
       <c r="K35" t="n">
-        <v>0.895833</v>
+        <v>0.77</v>
       </c>
       <c r="L35" t="n">
-        <v>0.886598</v>
+        <v>0.793814</v>
       </c>
       <c r="M35" t="n">
-        <v>0.891192</v>
+        <v>0.781726</v>
       </c>
       <c r="N35" t="n">
         <v>0.2</v>
@@ -3985,7 +3985,7 @@
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>_4_10_1_1790733345_2.txt</t>
+          <t>_4_10_1_1790733345_13.txt</t>
         </is>
       </c>
       <c r="Y35" t="inlineStr">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="AC35" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -4015,7 +4015,7 @@
         <v>0.1</v>
       </c>
       <c r="B36" t="n">
-        <v>0.134268</v>
+        <v>0.131362</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -4032,25 +4032,25 @@
         <v>200000</v>
       </c>
       <c r="G36" t="n">
-        <v>0.800971</v>
+        <v>0.812958</v>
       </c>
       <c r="H36" t="n">
-        <v>0.816832</v>
+        <v>0.82302</v>
       </c>
       <c r="I36" t="n">
-        <v>0.808823</v>
+        <v>0.817958</v>
       </c>
       <c r="J36" t="n">
-        <v>0.141901</v>
+        <v>0.136797</v>
       </c>
       <c r="K36" t="n">
-        <v>0.780749</v>
+        <v>0.796791</v>
       </c>
       <c r="L36" t="n">
-        <v>0.7525770000000001</v>
+        <v>0.768041</v>
       </c>
       <c r="M36" t="n">
-        <v>0.766404</v>
+        <v>0.782152</v>
       </c>
       <c r="N36" t="n">
         <v>0.2</v>
@@ -4086,7 +4086,7 @@
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>_4_10_1_1790733345_19.txt</t>
+          <t>_4_10_1_1790733345_18.txt</t>
         </is>
       </c>
       <c r="Y36" t="inlineStr">
@@ -4116,42 +4116,42 @@
         <v>0.1</v>
       </c>
       <c r="B37" t="n">
-        <v>0.210196</v>
+        <v>0.09220200000000001</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>_4_5_5_1_</t>
+          <t>_4_10_1_</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1790733397</v>
+        <v>1790733345</v>
       </c>
       <c r="E37" t="n">
-        <v>89</v>
+        <v>52</v>
       </c>
       <c r="F37" t="n">
         <v>200000</v>
       </c>
       <c r="G37" t="n">
-        <v>0.666253</v>
+        <v>0.907006</v>
       </c>
       <c r="H37" t="n">
-        <v>0.664604</v>
+        <v>0.881188</v>
       </c>
       <c r="I37" t="n">
-        <v>0.665428</v>
+        <v>0.893911</v>
       </c>
       <c r="J37" t="n">
-        <v>0.205773</v>
+        <v>0.097304</v>
       </c>
       <c r="K37" t="n">
-        <v>0.6769230000000001</v>
+        <v>0.862069</v>
       </c>
       <c r="L37" t="n">
-        <v>0.680412</v>
+        <v>0.902062</v>
       </c>
       <c r="M37" t="n">
-        <v>0.678663</v>
+        <v>0.881612</v>
       </c>
       <c r="N37" t="n">
         <v>0.2</v>
@@ -4187,28 +4187,28 @@
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>_4_5_5_1_1790733397_2.txt</t>
+          <t>_4_10_1_1790733345_5.txt</t>
         </is>
       </c>
       <c r="Y37" t="inlineStr">
         <is>
-          <t>[5, 5]</t>
+          <t>[10]</t>
         </is>
       </c>
       <c r="Z37" t="n">
         <v>10</v>
       </c>
       <c r="AA37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB37" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC37" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Si</t>
         </is>
       </c>
     </row>
@@ -4217,42 +4217,42 @@
         <v>0.1</v>
       </c>
       <c r="B38" t="n">
-        <v>0.22867</v>
+        <v>0.129223</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>_4_5_5_1_</t>
+          <t>_4_10_1_</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>1790733397</v>
+        <v>1790733345</v>
       </c>
       <c r="E38" t="n">
-        <v>89</v>
+        <v>52</v>
       </c>
       <c r="F38" t="n">
         <v>200000</v>
       </c>
       <c r="G38" t="n">
-        <v>0.655797</v>
+        <v>0.805861</v>
       </c>
       <c r="H38" t="n">
-        <v>0.67203</v>
+        <v>0.816832</v>
       </c>
       <c r="I38" t="n">
-        <v>0.663814</v>
+        <v>0.8113089999999999</v>
       </c>
       <c r="J38" t="n">
-        <v>0.229602</v>
+        <v>0.141638</v>
       </c>
       <c r="K38" t="n">
-        <v>0.625592</v>
+        <v>0.765854</v>
       </c>
       <c r="L38" t="n">
-        <v>0.680412</v>
+        <v>0.8092780000000001</v>
       </c>
       <c r="M38" t="n">
-        <v>0.651852</v>
+        <v>0.786967</v>
       </c>
       <c r="N38" t="n">
         <v>0.2</v>
@@ -4288,23 +4288,23 @@
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>_4_5_5_1_1790733397_11.txt</t>
+          <t>_4_10_1_1790733345_0.txt</t>
         </is>
       </c>
       <c r="Y38" t="inlineStr">
         <is>
-          <t>[5, 5]</t>
+          <t>[10]</t>
         </is>
       </c>
       <c r="Z38" t="n">
         <v>10</v>
       </c>
       <c r="AA38" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB38" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC38" t="inlineStr">
@@ -4318,42 +4318,42 @@
         <v>0.1</v>
       </c>
       <c r="B39" t="n">
-        <v>0.09220200000000001</v>
+        <v>0.248854</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>_4_10_1_</t>
+          <t>_4_5_5_1_</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>1790733345</v>
+        <v>1790733397</v>
       </c>
       <c r="E39" t="n">
-        <v>52</v>
+        <v>89</v>
       </c>
       <c r="F39" t="n">
         <v>200000</v>
       </c>
       <c r="G39" t="n">
-        <v>0.907006</v>
+        <v>0.550234</v>
       </c>
       <c r="H39" t="n">
-        <v>0.881188</v>
+        <v>0.582921</v>
       </c>
       <c r="I39" t="n">
-        <v>0.893911</v>
+        <v>0.566106</v>
       </c>
       <c r="J39" t="n">
-        <v>0.097304</v>
+        <v>0.251222</v>
       </c>
       <c r="K39" t="n">
-        <v>0.862069</v>
+        <v>0.509346</v>
       </c>
       <c r="L39" t="n">
-        <v>0.902062</v>
+        <v>0.561856</v>
       </c>
       <c r="M39" t="n">
-        <v>0.881612</v>
+        <v>0.534314</v>
       </c>
       <c r="N39" t="n">
         <v>0.2</v>
@@ -4389,28 +4389,28 @@
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>_4_10_1_1790733345_5.txt</t>
+          <t>_4_5_5_1_1790733397_18.txt</t>
         </is>
       </c>
       <c r="Y39" t="inlineStr">
         <is>
-          <t>[10]</t>
+          <t>[5, 5]</t>
         </is>
       </c>
       <c r="Z39" t="n">
         <v>10</v>
       </c>
       <c r="AA39" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB39" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC39" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -4419,42 +4419,42 @@
         <v>0.1</v>
       </c>
       <c r="B40" t="n">
-        <v>0.248854</v>
+        <v>0.121098</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>_4_5_5_1_</t>
+          <t>_4_10_1_</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>1790733397</v>
+        <v>1790733345</v>
       </c>
       <c r="E40" t="n">
-        <v>89</v>
+        <v>52</v>
       </c>
       <c r="F40" t="n">
         <v>200000</v>
       </c>
       <c r="G40" t="n">
-        <v>0.550234</v>
+        <v>0.826406</v>
       </c>
       <c r="H40" t="n">
-        <v>0.582921</v>
+        <v>0.836634</v>
       </c>
       <c r="I40" t="n">
-        <v>0.566106</v>
+        <v>0.831488</v>
       </c>
       <c r="J40" t="n">
-        <v>0.251222</v>
+        <v>0.131535</v>
       </c>
       <c r="K40" t="n">
-        <v>0.509346</v>
+        <v>0.808511</v>
       </c>
       <c r="L40" t="n">
-        <v>0.561856</v>
+        <v>0.783505</v>
       </c>
       <c r="M40" t="n">
-        <v>0.534314</v>
+        <v>0.795812</v>
       </c>
       <c r="N40" t="n">
         <v>0.2</v>
@@ -4490,23 +4490,23 @@
       </c>
       <c r="X40" t="inlineStr">
         <is>
-          <t>_4_5_5_1_1790733397_18.txt</t>
+          <t>_4_10_1_1790733345_15.txt</t>
         </is>
       </c>
       <c r="Y40" t="inlineStr">
         <is>
-          <t>[5, 5]</t>
+          <t>[10]</t>
         </is>
       </c>
       <c r="Z40" t="n">
         <v>10</v>
       </c>
       <c r="AA40" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB40" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC40" t="inlineStr">
@@ -4520,42 +4520,42 @@
         <v>0.1</v>
       </c>
       <c r="B41" t="n">
-        <v>0.093891</v>
+        <v>0.176646</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>_4_10_1_</t>
+          <t>_4_5_5_1_</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>1790733345</v>
+        <v>1790733397</v>
       </c>
       <c r="E41" t="n">
-        <v>52</v>
+        <v>89</v>
       </c>
       <c r="F41" t="n">
         <v>200000</v>
       </c>
       <c r="G41" t="n">
-        <v>0.877928</v>
+        <v>0.720253</v>
       </c>
       <c r="H41" t="n">
-        <v>0.881188</v>
+        <v>0.7042079999999999</v>
       </c>
       <c r="I41" t="n">
-        <v>0.879555</v>
+        <v>0.71214</v>
       </c>
       <c r="J41" t="n">
-        <v>0.104515</v>
+        <v>0.183729</v>
       </c>
       <c r="K41" t="n">
-        <v>0.831633</v>
+        <v>0.700565</v>
       </c>
       <c r="L41" t="n">
-        <v>0.840206</v>
+        <v>0.639175</v>
       </c>
       <c r="M41" t="n">
-        <v>0.835897</v>
+        <v>0.6684639999999999</v>
       </c>
       <c r="N41" t="n">
         <v>0.2</v>
@@ -4591,28 +4591,28 @@
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>_4_10_1_1790733345_9.txt</t>
+          <t>_4_5_5_1_1790733397_4.txt</t>
         </is>
       </c>
       <c r="Y41" t="inlineStr">
         <is>
-          <t>[10]</t>
+          <t>[5, 5]</t>
         </is>
       </c>
       <c r="Z41" t="n">
         <v>10</v>
       </c>
       <c r="AA41" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB41" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC41" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -4682,7 +4682,7 @@
         <v>0.80901675</v>
       </c>
       <c r="C2" t="n">
-        <v>0.04801426527373208</v>
+        <v>0.04801426527373207</v>
       </c>
       <c r="D2" t="n">
         <v>0.912467</v>
@@ -4710,7 +4710,7 @@
         <v>0.585058</v>
       </c>
       <c r="C3" t="n">
-        <v>0.07864027062985506</v>
+        <v>0.07864027062985507</v>
       </c>
       <c r="D3" t="n">
         <v>0.709524</v>

</xml_diff>